<commit_message>
added Mann-Whitney U Test p-values for the parental-daughter copies to the distanceTable
</commit_message>
<xml_diff>
--- a/data/automatedDistancesWithRandomAndParentalDaughterCorr.xlsx
+++ b/data/automatedDistancesWithRandomAndParentalDaughterCorr.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="31">
   <si>
     <t>Category</t>
   </si>
@@ -104,10 +104,10 @@
     <t>trios, duplicated in human, parental</t>
   </si>
   <si>
-    <t>trios, duplicated in human, daughter</t>
+    <t>trios, duplicated in mouse, parental</t>
   </si>
   <si>
-    <t>trios, duplicated in mouse, parental</t>
+    <t>trios, duplicated in human, daughter</t>
   </si>
   <si>
     <t>trios, duplicated in mouse, daughter</t>
@@ -128,7 +128,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -160,18 +160,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="8">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
@@ -179,6 +170,9 @@
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -188,9 +182,6 @@
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -497,20 +488,20 @@
   <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="10" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="10" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="10" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="7" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -545,21 +536,21 @@
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="2">
         <v>16116</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="3">
         <v>45.77909218298488</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="3">
         <v>255.6504672975712</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1" t="s">
@@ -568,25 +559,25 @@
       <c r="J2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="6">
-        <v>1.350181665608108e-11</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
+      <c r="K2" s="3">
+        <v>1.3502e-11</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="2">
         <v>1886</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="3">
         <v>7.789615286549974</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="3">
         <v>461.5168731852765</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1" t="s">
@@ -595,27 +586,27 @@
       <c r="J3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="6">
+      <c r="K3" s="3">
         <v>3.637248062312788e-138</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="2">
         <v>480</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="3">
         <v>25.50348544312759</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="3">
         <v>1012.029178094124</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="3">
         <v>-0.1708519724980002</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="3">
         <v>0.0001691617538852674</v>
       </c>
       <c r="G4" s="1"/>
@@ -626,27 +617,27 @@
       <c r="J4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="3">
         <v>3.051560457160361e-11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="2">
         <v>221</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="3">
         <v>29.22451953055087</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="3">
         <v>393.9036352899958</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="3">
         <v>-0.02918675867562775</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="3">
         <v>0.6660875790546673</v>
       </c>
       <c r="G5" s="1"/>
@@ -657,27 +648,27 @@
       <c r="J5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="3">
         <v>1.507190226900653e-117</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="2">
         <v>46</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="3">
         <v>4.922672973558837</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="3">
         <v>82.4967793413032</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="3">
         <v>-0.2673723303404958</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="3">
         <v>0.07243674527966126</v>
       </c>
       <c r="G6" s="1"/>
@@ -688,27 +679,27 @@
       <c r="J6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="3">
         <v>1.910267034103454e-152</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="2">
         <v>69</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="3">
         <v>17.22795344153132</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="3">
         <v>72.08782489854175</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="3">
         <v>-0.3575114736916072</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="3">
         <v>0.002562928439554303</v>
       </c>
       <c r="G7" s="1"/>
@@ -719,27 +710,27 @@
       <c r="J7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="K7" s="6">
+      <c r="K7" s="3">
         <v>0.0091173679240049</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="2">
         <v>28</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="3">
         <v>23.07131030957849</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="3">
         <v>171.1032846516759</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="3">
         <v>-0.1789987104656345</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="3">
         <v>0.3620953450659865</v>
       </c>
       <c r="G8" s="1"/>
@@ -750,27 +741,27 @@
       <c r="J8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="6">
+      <c r="K8" s="3">
         <v>0.0505448337449901</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="2">
         <v>116</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="3">
         <v>49.90492511772983</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="3">
         <v>3320.357744380555</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="3">
         <v>-0.3432600995896886</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="3">
         <v>0.0001617689633040599</v>
       </c>
       <c r="G9" s="1"/>
@@ -781,27 +772,27 @@
       <c r="J9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K9" s="6">
+      <c r="K9" s="3">
         <v>0.9017924803746654</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="2">
         <v>1405</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="3">
         <v>5.020402966346215</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="3">
         <v>273.3271894648888</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="3">
         <v>-0.2134081188744889</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="3">
         <v>6.193750508727909e-16</v>
       </c>
       <c r="G10" s="1"/>
@@ -812,27 +803,27 @@
       <c r="J10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K10" s="6">
+      <c r="K10" s="3">
         <v>0.326203746787139</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="2">
         <v>567</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="3">
         <v>1.765445975351184</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="3">
         <v>142.361515099448</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="3">
         <v>-0.2931594438091105</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="3">
         <v>1.061320748719085e-12</v>
       </c>
       <c r="G11" s="1"/>
@@ -843,27 +834,27 @@
       <c r="J11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K11" s="6">
+      <c r="K11" s="3">
         <v>0.1398604668479114</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="2">
         <v>143</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="3">
         <v>0.1184066419388636</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="3">
         <v>692.6975540030611</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="3">
         <v>-0.08516169155465957</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="3">
         <v>0.3118794403998532</v>
       </c>
       <c r="G12" s="1"/>
@@ -874,27 +865,27 @@
       <c r="J12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="K12" s="6">
+      <c r="K12" s="3">
         <v>6.662261769554549e-9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="2">
         <v>198</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="3">
         <v>2.765075320770856</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="3">
         <v>83.05181805649485</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="3">
         <v>-0.1966957907611255</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="3">
         <v>0.005479298744152036</v>
       </c>
       <c r="G13" s="1"/>
@@ -905,27 +896,27 @@
       <c r="J13" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K13" s="6">
+      <c r="K13" s="3">
         <v>0.0228362099944615</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="2">
         <v>122</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="3">
         <v>0.0894696368333951</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="3">
         <v>165.4879370863909</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="3">
         <v>-0.3802672625534861</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="3">
         <v>0.00001557461267960093</v>
       </c>
       <c r="G14" s="1"/>
@@ -936,27 +927,27 @@
       <c r="J14" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="K14" s="6">
+      <c r="K14" s="3">
         <v>0.0530330052310332</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="2">
         <v>375</v>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="3">
         <v>37.14590489357546</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="3">
         <v>446.9764896389818</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="3">
         <v>0.0679625945725712</v>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="3">
         <v>0.1891104882001017</v>
       </c>
       <c r="G15" s="1"/>
@@ -967,25 +958,25 @@
       <c r="J15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K15" s="6">
+      <c r="K15" s="3">
         <v>1.105687979322487e-19</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="5">
+      <c r="B16" s="2">
         <v>3998</v>
       </c>
-      <c r="C16" s="6">
+      <c r="C16" s="3">
         <v>0.0339430432876772</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="3">
         <v>437.4838637315118</v>
       </c>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1" t="s">
@@ -994,114 +985,126 @@
       <c r="J16" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K16" s="6">
+      <c r="K16" s="3">
         <v>7.737169318639102e-19</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="5">
+      <c r="B17" s="2">
         <v>10000</v>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="3">
         <v>63.02235894190287</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="3">
         <v>349.6768238601636</v>
       </c>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18">
+      <c r="I17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K17" s="3">
+        <v>0.004692891533260526</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="5">
+      <c r="B18" s="2">
         <v>139</v>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="3">
         <v>30.09496872068533</v>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="3">
         <v>463.8818865814138</v>
       </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18">
+      <c r="I18" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="K18" s="3">
+        <v>6.287160245303312e-9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="5">
+        <v>29</v>
+      </c>
+      <c r="B19" s="2">
         <v>170</v>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="3">
         <v>51.22465067228259</v>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="3">
         <v>517.7826281804561</v>
       </c>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
-      <c r="K19" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18">
+      <c r="K19" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" s="5">
+        <v>28</v>
+      </c>
+      <c r="B20" s="2">
         <v>364</v>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="3">
         <v>11.39424894466966</v>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="3">
         <v>286.7984910207074</v>
       </c>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
-      <c r="K20" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18">
+      <c r="K20" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="5">
+      <c r="B21" s="2">
         <v>478</v>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="3">
         <v>2.426821134633891</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="3">
         <v>200.1950702348572</v>
       </c>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
-      <c r="K21" s="4"/>
+      <c r="K21" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1116,17 +1119,17 @@
   <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="10" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="10" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="10" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="7" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
@@ -1168,17 +1171,17 @@
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="2">
         <v>15889</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="3">
         <v>0.5314054052381022</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="3">
         <v>0.5824958756637905</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1" t="s">
@@ -1187,7 +1190,7 @@
       <c r="J2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="6">
+      <c r="K2" s="3">
         <v>2.378793542410633e-10</v>
       </c>
     </row>
@@ -1195,17 +1198,17 @@
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="2">
         <v>1209</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="3">
         <v>0.7234932892136435</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="3">
         <v>0.7501344236066786</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1" t="s">
@@ -1214,7 +1217,7 @@
       <c r="J3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="6">
+      <c r="K3" s="3">
         <v>1.500204868451264e-53</v>
       </c>
     </row>
@@ -1222,19 +1225,19 @@
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="2">
         <v>419</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="3">
         <v>0.6313495949555581</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="3">
         <v>0.7001022178718169</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="3">
         <v>0.1755700696536351</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="3">
         <v>0.0003048045950849422</v>
       </c>
       <c r="G4" s="1"/>
@@ -1245,7 +1248,7 @@
       <c r="J4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="3">
         <v>0.0002012770815528</v>
       </c>
     </row>
@@ -1253,19 +1256,19 @@
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="2">
         <v>185</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="3">
         <v>0.6721679194966002</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="3">
         <v>0.7450029973680323</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="3">
         <v>-0.006920697142484956</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="3">
         <v>0.925510508034243</v>
       </c>
       <c r="G5" s="1"/>
@@ -1276,7 +1279,7 @@
       <c r="J5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="3">
         <v>2.780478500934892e-22</v>
       </c>
     </row>
@@ -1284,19 +1287,19 @@
       <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="2">
         <v>36</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="3">
         <v>0.7053902017678588</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="3">
         <v>0.7630430036959254</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="3">
         <v>0.2365259676728071</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="3">
         <v>0.1648723025957013</v>
       </c>
       <c r="G6" s="1"/>
@@ -1307,7 +1310,7 @@
       <c r="J6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="3">
         <v>4.84275119978293e-16</v>
       </c>
     </row>
@@ -1315,19 +1318,19 @@
       <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="2">
         <v>65</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="3">
         <v>0.5677308351250281</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="3">
         <v>0.6486531535362393</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="3">
         <v>0.2980798262979403</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="3">
         <v>0.01587976496142841</v>
       </c>
       <c r="G7" s="1"/>
@@ -1338,7 +1341,7 @@
       <c r="J7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="K7" s="6">
+      <c r="K7" s="3">
         <v>0.910401993128528</v>
       </c>
     </row>
@@ -1346,19 +1349,19 @@
       <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="2">
         <v>25</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="3">
         <v>0.5151550066523226</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="3">
         <v>0.5867420255282432</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="3">
         <v>-0.2402422655442755</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="3">
         <v>0.2473732088380338</v>
       </c>
       <c r="G8" s="1"/>
@@ -1369,7 +1372,7 @@
       <c r="J8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="6">
+      <c r="K8" s="3">
         <v>0.1722721250161584</v>
       </c>
     </row>
@@ -1377,19 +1380,19 @@
       <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="2">
         <v>108</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="3">
         <v>0.6006702772833892</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="3">
         <v>0.6594140835563914</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="3">
         <v>0.3358297918030919</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="3">
         <v>0.000380559362663576</v>
       </c>
       <c r="G9" s="1"/>
@@ -1400,7 +1403,7 @@
       <c r="J9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K9" s="6">
+      <c r="K9" s="3">
         <v>0.3442136833709817</v>
       </c>
     </row>
@@ -1408,19 +1411,19 @@
       <c r="A10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="2">
         <v>789</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="3">
         <v>0.7635629503484532</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="3">
         <v>0.7771711558054761</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="3">
         <v>0.189600234199377</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="3">
         <v>8.049744435662803e-8</v>
       </c>
       <c r="G10" s="1"/>
@@ -1431,7 +1434,7 @@
       <c r="J10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K10" s="6">
+      <c r="K10" s="3">
         <v>0.4217443491141769</v>
       </c>
     </row>
@@ -1439,19 +1442,19 @@
       <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="2">
         <v>259</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="3">
         <v>0.8114848523049711</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="3">
         <v>0.8310194729211502</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="3">
         <v>0.1453733895941109</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="3">
         <v>0.01924790152384017</v>
       </c>
       <c r="G11" s="1"/>
@@ -1462,7 +1465,7 @@
       <c r="J11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K11" s="6">
+      <c r="K11" s="3">
         <v>0.0653195441326496</v>
       </c>
     </row>
@@ -1470,19 +1473,19 @@
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="2">
         <v>57</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="3">
         <v>0.7658969341096828</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="3">
         <v>0.7663304487899996</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="3">
         <v>0.02029469713760541</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="3">
         <v>0.880888946648062</v>
       </c>
       <c r="G12" s="1"/>
@@ -1493,7 +1496,7 @@
       <c r="J12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="K12" s="6">
+      <c r="K12" s="3">
         <v>0.2322536140360831</v>
       </c>
     </row>
@@ -1501,19 +1504,19 @@
       <c r="A13" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="2">
         <v>103</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="3">
         <v>0.8590955430112233</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="3">
         <v>0.8251332979170943</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="3">
         <v>0.2593856483996914</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="3">
         <v>0.008149899644154208</v>
       </c>
       <c r="G13" s="1"/>
@@ -1524,7 +1527,7 @@
       <c r="J13" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K13" s="6">
+      <c r="K13" s="3">
         <v>0.3324690855232217</v>
       </c>
     </row>
@@ -1532,19 +1535,19 @@
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="2">
         <v>52</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="3">
         <v>0.7272534679835447</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="3">
         <v>0.716228709341451</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="3">
         <v>0.02903364668967899</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="3">
         <v>0.8381048789806296</v>
       </c>
       <c r="G14" s="1"/>
@@ -1555,7 +1558,7 @@
       <c r="J14" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="K14" s="6">
+      <c r="K14" s="3">
         <v>0.059377041853093</v>
       </c>
     </row>
@@ -1563,19 +1566,19 @@
       <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="2">
         <v>318</v>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="3">
         <v>0.6695976743701387</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="3">
         <v>0.7296872336216872</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="3">
         <v>0.1800613679151337</v>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="3">
         <v>0.001261020801355822</v>
       </c>
       <c r="G15" s="1"/>
@@ -1586,7 +1589,7 @@
       <c r="J15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K15" s="6">
+      <c r="K15" s="3">
         <v>0.9414673907802696</v>
       </c>
     </row>
@@ -1594,17 +1597,17 @@
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="5">
+      <c r="B16" s="2">
         <v>1179</v>
       </c>
-      <c r="C16" s="6">
+      <c r="C16" s="3">
         <v>0.9658006333661328</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="3">
         <v>0.9048385383822672</v>
       </c>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1" t="s">
@@ -1613,7 +1616,7 @@
       <c r="J16" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K16" s="6">
+      <c r="K16" s="3">
         <v>0.0010297283120043</v>
       </c>
     </row>
@@ -1621,106 +1624,118 @@
       <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="5">
+      <c r="B17" s="2">
         <v>8815</v>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="3">
         <v>0.8605867285197175</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="3">
         <v>0.8556209204684726</v>
       </c>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="4"/>
+      <c r="I17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K17" s="3">
+        <v>0.5359179256569138</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18">
       <c r="A18" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="5">
+      <c r="B18" s="2">
         <v>124</v>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="3">
         <v>0.5877780190343305</v>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="3">
         <v>0.6926386320246581</v>
       </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="4"/>
+      <c r="I18" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="K18" s="3">
+        <v>0.0004293534935965329</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18">
       <c r="A19" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="5">
+        <v>29</v>
+      </c>
+      <c r="B19" s="2">
         <v>147</v>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="3">
         <v>0.6148266589887761</v>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="3">
         <v>0.7005598416078963</v>
       </c>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
-      <c r="K19" s="4"/>
+      <c r="K19" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18">
       <c r="A20" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" s="5">
+        <v>28</v>
+      </c>
+      <c r="B20" s="2">
         <v>228</v>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="3">
         <v>0.5883025337642822</v>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="3">
         <v>0.6518375650698685</v>
       </c>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
-      <c r="K20" s="4"/>
+      <c r="K20" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18">
       <c r="A21" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="5">
+      <c r="B21" s="2">
         <v>207</v>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="3">
         <v>0.8147384789333834</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="3">
         <v>0.8255236950467534</v>
       </c>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
-      <c r="K21" s="4"/>
+      <c r="K21" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1735,17 +1750,17 @@
   <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="10" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="10" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="10" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="7" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
@@ -1787,17 +1802,17 @@
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="2">
         <v>16116</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="3">
         <v>3.627860650137308</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="3">
         <v>3.884749376566845</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1" t="s">
@@ -1806,7 +1821,7 @@
       <c r="J2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="6">
+      <c r="K2" s="3">
         <v>0.2219372643263294</v>
       </c>
     </row>
@@ -1814,17 +1829,17 @@
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="2">
         <v>1886</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="3">
         <v>2.657598392910077</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="3">
         <v>4.198831601081369</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1" t="s">
@@ -1833,7 +1848,7 @@
       <c r="J3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="6">
+      <c r="K3" s="3">
         <v>2.707094468845077e-38</v>
       </c>
     </row>
@@ -1841,19 +1856,19 @@
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="2">
         <v>480</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="3">
         <v>3.873037375023782</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="3">
         <v>5.24185444915052</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="3">
         <v>-0.1089000455322758</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="3">
         <v>0.01699749460364713</v>
       </c>
       <c r="G4" s="1"/>
@@ -1864,7 +1879,7 @@
       <c r="J4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="3">
         <v>1.093840151512434e-10</v>
       </c>
     </row>
@@ -1872,19 +1887,19 @@
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="2">
         <v>221</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="3">
         <v>4.684802360467556</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="3">
         <v>6.38449484139463</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="3">
         <v>0.009128312832021077</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="3">
         <v>0.8926629615617862</v>
       </c>
       <c r="G5" s="1"/>
@@ -1895,7 +1910,7 @@
       <c r="J5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="3">
         <v>7.298282127955101e-112</v>
       </c>
     </row>
@@ -1903,19 +1918,19 @@
       <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="2">
         <v>46</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="3">
         <v>2.887852143937579</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="3">
         <v>3.869523215535065</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="3">
         <v>-0.2528972015766168</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="3">
         <v>0.08993957234310268</v>
       </c>
       <c r="G6" s="1"/>
@@ -1926,7 +1941,7 @@
       <c r="J6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="3">
         <v>1.773415297715097e-144</v>
       </c>
     </row>
@@ -1934,19 +1949,19 @@
       <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="2">
         <v>69</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="3">
         <v>3.852696142984284</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="3">
         <v>4.642019179274294</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="3">
         <v>-0.3663924894835816</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="3">
         <v>0.001959370653549534</v>
       </c>
       <c r="G7" s="1"/>
@@ -1957,7 +1972,7 @@
       <c r="J7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="K7" s="6">
+      <c r="K7" s="3">
         <v>0.0116135561563776</v>
       </c>
     </row>
@@ -1965,19 +1980,19 @@
       <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="2">
         <v>28</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="3">
         <v>3.163807341684167</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="3">
         <v>3.858422140468076</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="3">
         <v>-0.2487092635364218</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="3">
         <v>0.2018812810577265</v>
       </c>
       <c r="G8" s="1"/>
@@ -1988,7 +2003,7 @@
       <c r="J8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="6">
+      <c r="K8" s="3">
         <v>0.1526888014319976</v>
       </c>
     </row>
@@ -1996,19 +2011,19 @@
       <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="2">
         <v>116</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="3">
         <v>3.554521511826952</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="3">
         <v>4.299858314020614</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="3">
         <v>-0.3515326962353558</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="3">
         <v>0.0001091171156070439</v>
       </c>
       <c r="G9" s="1"/>
@@ -2019,7 +2034,7 @@
       <c r="J9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K9" s="6">
+      <c r="K9" s="3">
         <v>0.3216078951232134</v>
       </c>
     </row>
@@ -2027,19 +2042,19 @@
       <c r="A10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="2">
         <v>1405</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="3">
         <v>2.199124880714502</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="3">
         <v>3.84059933491433</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="3">
         <v>-0.1449667119054401</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="3">
         <v>4.819268024926837e-8</v>
       </c>
       <c r="G10" s="1"/>
@@ -2050,7 +2065,7 @@
       <c r="J10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K10" s="6">
+      <c r="K10" s="3">
         <v>0.5908626675201291</v>
       </c>
     </row>
@@ -2058,19 +2073,19 @@
       <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="2">
         <v>567</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="3">
         <v>1.576167850372097</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="3">
         <v>4.281041457228843</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="3">
         <v>-0.277264196932519</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="3">
         <v>1.82016311562745e-11</v>
       </c>
       <c r="G11" s="1"/>
@@ -2081,7 +2096,7 @@
       <c r="J11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K11" s="6">
+      <c r="K11" s="3">
         <v>0.031973630220929</v>
       </c>
     </row>
@@ -2089,19 +2104,19 @@
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="2">
         <v>143</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="3">
         <v>0.1576244659695413</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="3">
         <v>2.286096050404656</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="3">
         <v>-0.04714464005863003</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="3">
         <v>0.5760723418710505</v>
       </c>
       <c r="G12" s="1"/>
@@ -2112,7 +2127,7 @@
       <c r="J12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="K12" s="6">
+      <c r="K12" s="3">
         <v>1.150105460269036e-9</v>
       </c>
     </row>
@@ -2120,19 +2135,19 @@
       <c r="A13" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="2">
         <v>198</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="3">
         <v>1.801459178879421</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="3">
         <v>3.367331144281187</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="3">
         <v>-0.1492639442847999</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="3">
         <v>0.03583421808878428</v>
       </c>
       <c r="G13" s="1"/>
@@ -2143,7 +2158,7 @@
       <c r="J13" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K13" s="6">
+      <c r="K13" s="3">
         <v>0.0263849660154784</v>
       </c>
     </row>
@@ -2151,19 +2166,19 @@
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="2">
         <v>122</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="3">
         <v>0.1178568994448193</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="3">
         <v>2.172869947086347</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="3">
         <v>-0.3584945943616073</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="3">
         <v>0.00005022995457379572</v>
       </c>
       <c r="G14" s="1"/>
@@ -2174,7 +2189,7 @@
       <c r="J14" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="K14" s="6">
+      <c r="K14" s="3">
         <v>0.022138076733667</v>
       </c>
     </row>
@@ -2182,19 +2197,19 @@
       <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="2">
         <v>375</v>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="3">
         <v>3.632491783498349</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="3">
         <v>4.559888330628813</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="3">
         <v>0.1681135174981331</v>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="3">
         <v>0.001083394479456426</v>
       </c>
       <c r="G15" s="1"/>
@@ -2205,7 +2220,7 @@
       <c r="J15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K15" s="6">
+      <c r="K15" s="3">
         <v>9.917558849787478e-16</v>
       </c>
     </row>
@@ -2213,17 +2228,17 @@
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="5">
+      <c r="B16" s="2">
         <v>3998</v>
       </c>
-      <c r="C16" s="6">
+      <c r="C16" s="3">
         <v>0.0472251677689699</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="3">
         <v>1.26377785272589</v>
       </c>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1" t="s">
@@ -2232,7 +2247,7 @@
       <c r="J16" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K16" s="6">
+      <c r="K16" s="3">
         <v>0.0003604277298871</v>
       </c>
     </row>
@@ -2240,106 +2255,118 @@
       <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="5">
+      <c r="B17" s="2">
         <v>10000</v>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="3">
         <v>6.944263591666727</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="3">
         <v>7.501727698817689</v>
       </c>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="4"/>
+      <c r="I17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K17" s="3">
+        <v>0.003617558505736715</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18">
       <c r="A18" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="5">
+      <c r="B18" s="2">
         <v>139</v>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="3">
         <v>3.593655738933193</v>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="3">
         <v>4.030228669613347</v>
       </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="4"/>
+      <c r="I18" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="K18" s="3">
+        <v>1.319358793955837e-7</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18">
       <c r="A19" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="5">
+        <v>29</v>
+      </c>
+      <c r="B19" s="2">
         <v>170</v>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="3">
         <v>6.495496770705548</v>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="3">
         <v>7.299733697536823</v>
       </c>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
-      <c r="K19" s="4"/>
+      <c r="K19" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18">
       <c r="A20" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" s="5">
+        <v>28</v>
+      </c>
+      <c r="B20" s="2">
         <v>364</v>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="3">
         <v>2.454846358371422</v>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="3">
         <v>3.579622080851999</v>
       </c>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
-      <c r="K20" s="4"/>
+      <c r="K20" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18">
       <c r="A21" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="5">
+      <c r="B21" s="2">
         <v>478</v>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="3">
         <v>1.887883976951877</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="3">
         <v>4.607737962641218</v>
       </c>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
-      <c r="K21" s="4"/>
+      <c r="K21" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2354,17 +2381,17 @@
   <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="10" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="10" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="10" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="7" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
@@ -2406,17 +2433,17 @@
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="2">
         <v>15889</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="3">
         <v>0.4805531078119407</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="3">
         <v>0.5259569721865671</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1" t="s">
@@ -2425,7 +2452,7 @@
       <c r="J2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="6">
+      <c r="K2" s="3">
         <v>5.992501964104844e-14</v>
       </c>
     </row>
@@ -2433,17 +2460,17 @@
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="2">
         <v>1209</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="3">
         <v>0.6966403113785433</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="3">
         <v>0.6929805072595744</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1" t="s">
@@ -2452,7 +2479,7 @@
       <c r="J3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="6">
+      <c r="K3" s="3">
         <v>5.154371641200041e-29</v>
       </c>
     </row>
@@ -2460,19 +2487,19 @@
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="2">
         <v>419</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="3">
         <v>0.6944367014933688</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="3">
         <v>0.6859136353268297</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="3">
         <v>0.1757200910270652</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="3">
         <v>0.0003011408567441984</v>
       </c>
       <c r="G4" s="1"/>
@@ -2483,7 +2510,7 @@
       <c r="J4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="3">
         <v>0.6064538603804193</v>
       </c>
     </row>
@@ -2491,19 +2518,19 @@
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="2">
         <v>185</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="3">
         <v>0.7472474236155728</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="3">
         <v>0.7724969578623798</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="3">
         <v>0.06346641379509176</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="3">
         <v>0.3907537065822809</v>
       </c>
       <c r="G5" s="1"/>
@@ -2514,7 +2541,7 @@
       <c r="J5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="3">
         <v>0.000004225349748574983</v>
       </c>
     </row>
@@ -2522,19 +2549,19 @@
       <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="2">
         <v>36</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="3">
         <v>0.7422452056922164</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="3">
         <v>0.7295485588029825</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="3">
         <v>0.2524715385271536</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="3">
         <v>0.1373969593593788</v>
       </c>
       <c r="G6" s="1"/>
@@ -2545,7 +2572,7 @@
       <c r="J6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="3">
         <v>1.793814010954497e-7</v>
       </c>
     </row>
@@ -2553,19 +2580,19 @@
       <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="2">
         <v>65</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="3">
         <v>0.5877335531781513</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="3">
         <v>0.6128270826550761</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="3">
         <v>0.1340528090924358</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="3">
         <v>0.2870515514505487</v>
       </c>
       <c r="G7" s="1"/>
@@ -2576,7 +2603,7 @@
       <c r="J7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="K7" s="6">
+      <c r="K7" s="3">
         <v>0.7768200782669609</v>
       </c>
     </row>
@@ -2584,19 +2611,19 @@
       <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="2">
         <v>25</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="3">
         <v>0.5408664349045855</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="3">
         <v>0.5451387005088786</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="3">
         <v>-0.1209382833352135</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="3">
         <v>0.5647139524424951</v>
       </c>
       <c r="G8" s="1"/>
@@ -2607,7 +2634,7 @@
       <c r="J8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="6">
+      <c r="K8" s="3">
         <v>0.2266834967264824</v>
       </c>
     </row>
@@ -2615,19 +2642,19 @@
       <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="2">
         <v>108</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="3">
         <v>0.6513305373373708</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="3">
         <v>0.599628703659186</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="3">
         <v>0.2654950980685856</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="3">
         <v>0.005485947426035406</v>
       </c>
       <c r="G9" s="1"/>
@@ -2638,7 +2665,7 @@
       <c r="J9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K9" s="6">
+      <c r="K9" s="3">
         <v>0.3629073471073104</v>
       </c>
     </row>
@@ -2646,19 +2673,19 @@
       <c r="A10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="2">
         <v>789</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="3">
         <v>0.7010632237999191</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="3">
         <v>0.6974940184252307</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="3">
         <v>0.1668518206910886</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="3">
         <v>0.000002448575308503393</v>
       </c>
       <c r="G10" s="1"/>
@@ -2669,7 +2696,7 @@
       <c r="J10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K10" s="6">
+      <c r="K10" s="3">
         <v>0.723199115516034</v>
       </c>
     </row>
@@ -2677,19 +2704,19 @@
       <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="2">
         <v>259</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="3">
         <v>0.8226892256651179</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="3">
         <v>0.7750447157571532</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="3">
         <v>0.1762509341932775</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="3">
         <v>0.004440080354473454</v>
       </c>
       <c r="G11" s="1"/>
@@ -2700,7 +2727,7 @@
       <c r="J11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K11" s="6">
+      <c r="K11" s="3">
         <v>0.0022606026914326</v>
       </c>
     </row>
@@ -2708,19 +2735,19 @@
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="2">
         <v>57</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="3">
         <v>0.7606902079922337</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="3">
         <v>0.7235832673313256</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="3">
         <v>0.318104503668264</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="3">
         <v>0.01589001350252763</v>
       </c>
       <c r="G12" s="1"/>
@@ -2731,7 +2758,7 @@
       <c r="J12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="K12" s="6">
+      <c r="K12" s="3">
         <v>0.37071805725904</v>
       </c>
     </row>
@@ -2739,19 +2766,19 @@
       <c r="A13" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="2">
         <v>103</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="3">
         <v>0.8177963589251355</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="3">
         <v>0.7623146515521545</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="3">
         <v>0.2804078793633772</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="3">
         <v>0.004119146186644307</v>
       </c>
       <c r="G13" s="1"/>
@@ -2762,7 +2789,7 @@
       <c r="J13" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K13" s="6">
+      <c r="K13" s="3">
         <v>0.549443805619761</v>
       </c>
     </row>
@@ -2770,19 +2797,19 @@
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="2">
         <v>52</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="3">
         <v>0.5457292491951884</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="3">
         <v>0.6471940710108911</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="3">
         <v>0.01766850209733754</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="3">
         <v>0.9010604707677002</v>
       </c>
       <c r="G14" s="1"/>
@@ -2793,7 +2820,7 @@
       <c r="J14" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="K14" s="6">
+      <c r="K14" s="3">
         <v>0.0877714222874824</v>
       </c>
     </row>
@@ -2801,19 +2828,19 @@
       <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="2">
         <v>318</v>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="3">
         <v>0.6088205474002405</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="3">
         <v>0.6168850695474231</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="3">
         <v>0.03810037227900302</v>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="3">
         <v>0.498407683538053</v>
       </c>
       <c r="G15" s="1"/>
@@ -2824,7 +2851,7 @@
       <c r="J15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K15" s="6">
+      <c r="K15" s="3">
         <v>0.7292302979458066</v>
       </c>
     </row>
@@ -2832,17 +2859,17 @@
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="5">
+      <c r="B16" s="2">
         <v>1179</v>
       </c>
-      <c r="C16" s="6">
+      <c r="C16" s="3">
         <v>0.8936126372781039</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="3">
         <v>0.7982190398504989</v>
       </c>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1" t="s">
@@ -2851,7 +2878,7 @@
       <c r="J16" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K16" s="6">
+      <c r="K16" s="3">
         <v>0.000008952076089975636</v>
       </c>
     </row>
@@ -2859,106 +2886,118 @@
       <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="5">
+      <c r="B17" s="2">
         <v>8815</v>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="3">
         <v>0.85262850002279</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="3">
         <v>0.8339085493085807</v>
       </c>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="4"/>
+      <c r="I17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K17" s="3">
+        <v>0.209084002382087</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18">
       <c r="A18" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="5">
+      <c r="B18" s="2">
         <v>124</v>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="3">
         <v>0.6986355140505016</v>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="3">
         <v>0.6694691498857065</v>
       </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="4"/>
+      <c r="I18" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="K18" s="3">
+        <v>0.9118796242072658</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18">
       <c r="A19" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="5">
+        <v>29</v>
+      </c>
+      <c r="B19" s="2">
         <v>147</v>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="3">
         <v>0.7255156351339915</v>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="3">
         <v>0.7301413887235658</v>
       </c>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
-      <c r="K19" s="4"/>
+      <c r="K19" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18">
       <c r="A20" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" s="5">
+        <v>28</v>
+      </c>
+      <c r="B20" s="2">
         <v>228</v>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="3">
         <v>0.6146966692894987</v>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="3">
         <v>0.6086576774153598</v>
       </c>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
-      <c r="K20" s="4"/>
+      <c r="K20" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18">
       <c r="A21" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="5">
+      <c r="B21" s="2">
         <v>207</v>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="3">
         <v>0.7739633854494103</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="3">
         <v>0.7383899456024707</v>
       </c>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
-      <c r="K21" s="4"/>
+      <c r="K21" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2973,17 +3012,17 @@
   <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="10" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="10" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="10" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="7" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="7" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
@@ -3021,21 +3060,21 @@
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="2">
         <v>14186</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="3">
         <v>0.0625</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="3">
         <v>0.1094397645566051</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1" t="s">
@@ -3044,25 +3083,25 @@
       <c r="J2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="6">
+      <c r="K2" s="3">
         <v>3.081682612439242e-7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="2">
         <v>696</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="3">
         <v>0.125</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="3">
         <v>0.2210163519430761</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1" t="s">
@@ -3071,27 +3110,27 @@
       <c r="J3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="6">
+      <c r="K3" s="3">
         <v>4.020786444740382e-33</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="2">
         <v>217</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="3">
         <v>0.0625</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="3">
         <v>0.218556616194865</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="3">
         <v>0.03593152046540014</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="3">
         <v>0.5985983096240637</v>
       </c>
       <c r="G4" s="1"/>
@@ -3102,27 +3141,27 @@
       <c r="J4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="3">
         <v>0.0821386061510113</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="2">
         <v>69</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="3">
         <v>0.125</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="3">
         <v>0.2609126984126984</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="3">
         <v>-0.09177318628061466</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="3">
         <v>0.4532647685490119</v>
       </c>
       <c r="G5" s="1"/>
@@ -3133,27 +3172,27 @@
       <c r="J5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="3">
         <v>3.513036444740924e-8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="2">
         <v>18</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="3">
         <v>0.225</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="3">
         <v>0.2967261904761905</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="3">
         <v>0.4260012232700152</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="3">
         <v>0.07794629372125841</v>
       </c>
       <c r="G6" s="1"/>
@@ -3164,27 +3203,27 @@
       <c r="J6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="3">
         <v>2.180152254364907e-7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="2">
         <v>42</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="3">
         <v>0.1339285714285714</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="3">
         <v>0.2232993197278911</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="3">
         <v>0.2717875933039477</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="3">
         <v>0.08165342274398779</v>
       </c>
       <c r="G7" s="1"/>
@@ -3195,27 +3234,27 @@
       <c r="J7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="K7" s="6">
+      <c r="K7" s="3">
         <v>0.2848874864143457</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="2">
         <v>19</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="3">
         <v>0.0625</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="3">
         <v>0.1371553884711779</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="3">
         <v>-0.3309943796164508</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="3">
         <v>0.166293936663228</v>
       </c>
       <c r="G8" s="1"/>
@@ -3226,27 +3265,27 @@
       <c r="J8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="6">
+      <c r="K8" s="3">
         <v>0.4191112239150441</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="2">
         <v>69</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="3">
         <v>0.0625</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="3">
         <v>0.1753364389233954</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="3">
         <v>-0.1191804196703512</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="3">
         <v>0.3293702946111322</v>
       </c>
       <c r="G9" s="1"/>
@@ -3257,27 +3296,27 @@
       <c r="J9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K9" s="6">
+      <c r="K9" s="3">
         <v>0.0928225185254886</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="2">
         <v>478</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="3">
         <v>0.1428571428571428</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="3">
         <v>0.2224646343893205</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="3">
         <v>0.2316330327835759</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="3">
         <v>3.042594924252342e-7</v>
       </c>
       <c r="G10" s="1"/>
@@ -3288,27 +3327,27 @@
       <c r="J10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K10" s="6">
+      <c r="K10" s="3">
         <v>0.7640876022274787</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="2">
         <v>104</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="3">
         <v>0.25</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="3">
         <v>0.2775526556776556</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="3">
         <v>-0.03263457486948008</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="3">
         <v>0.7422510109786792</v>
       </c>
       <c r="G11" s="1"/>
@@ -3319,27 +3358,27 @@
       <c r="J11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K11" s="6">
+      <c r="K11" s="3">
         <v>0.2029809474210726</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="2">
         <v>37</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="3">
         <v>0.1875</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="3">
         <v>0.2339124839124839</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="3">
         <v>-0.3303335047718227</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="3">
         <v>0.04584435677962395</v>
       </c>
       <c r="G12" s="1"/>
@@ -3350,27 +3389,27 @@
       <c r="J12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="K12" s="6">
+      <c r="K12" s="3">
         <v>0.2952375065759116</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="2">
         <v>63</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="3">
         <v>0.1875</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="3">
         <v>0.2554421768707482</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="3">
         <v>0.1534205254732786</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="3">
         <v>0.2299548915527978</v>
       </c>
       <c r="G13" s="1"/>
@@ -3381,27 +3420,27 @@
       <c r="J13" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K13" s="6">
+      <c r="K13" s="3">
         <v>0.8599529172108156</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="2">
         <v>37</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="3">
         <v>0.1875</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="3">
         <v>0.2224903474903475</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="3">
         <v>0.3477455314100384</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="3">
         <v>0.03494685870057278</v>
       </c>
       <c r="G14" s="1"/>
@@ -3412,27 +3451,27 @@
       <c r="J14" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="K14" s="6">
+      <c r="K14" s="3">
         <v>0.6972780044974736</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="2">
         <v>237</v>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="3">
         <v>0.0714285714285714</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="3">
         <v>0.1877335744424351</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="3">
         <v>0.3717133887064786</v>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="3">
         <v>3.523374472307563e-9</v>
       </c>
       <c r="G15" s="1"/>
@@ -3443,25 +3482,25 @@
       <c r="J15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K15" s="6">
+      <c r="K15" s="3">
         <v>0.2054737725398945</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="5">
+      <c r="B16" s="2">
         <v>387</v>
       </c>
-      <c r="C16" s="6">
+      <c r="C16" s="3">
         <v>0.25</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="3">
         <v>0.3144825889011935</v>
       </c>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1" t="s">
@@ -3470,114 +3509,126 @@
       <c r="J16" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K16" s="6">
+      <c r="K16" s="3">
         <v>0.0002196991850601</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="5">
+      <c r="B17" s="2">
         <v>6822</v>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="3">
         <v>0.125</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="3">
         <v>0.2005028374586422</v>
       </c>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18">
+      <c r="I17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K17" s="3">
+        <v>0.6782776898861298</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="5">
+      <c r="B18" s="2">
         <v>89</v>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="3">
         <v>0.0625</v>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="3">
         <v>0.1900147137506688</v>
       </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18">
+      <c r="I18" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="K18" s="3">
+        <v>0.6160928633805518</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="5">
+        <v>29</v>
+      </c>
+      <c r="B19" s="2">
         <v>57</v>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="3">
         <v>0.2857142857142857</v>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="3">
         <v>0.3076545530492898</v>
       </c>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
-      <c r="K19" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18">
+      <c r="K19" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" s="5">
+        <v>28</v>
+      </c>
+      <c r="B20" s="2">
         <v>166</v>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="3">
         <v>0.0625</v>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="3">
         <v>0.1305507745266781</v>
       </c>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
-      <c r="K20" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18">
+      <c r="K20" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="5">
+      <c r="B21" s="2">
         <v>88</v>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="3">
         <v>0.25</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="3">
         <v>0.2638257575757575</v>
       </c>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
-      <c r="K21" s="4"/>
+      <c r="K21" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>